<commit_message>
feat: Enable eager change detection strategy for multiple components - Modified HTML templates to utilize safe navigation for optional properties in purchase and sales order invoices. - Added new ProductUpload.xlsx file and updated Chemicals.xlsx.
</commit_message>
<xml_diff>
--- a/src/assets/csv/Chemicals.xlsx
+++ b/src/assets/csv/Chemicals.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Software\Projects\Chem4Buy\chem4buyadmin\src\assets\csv\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\jaydip\Jigs Chemical\jigschemicalsadmin\src\assets\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C022254-28C6-4C20-A158-49897875B8BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330"/>
+    <workbookView xWindow="7200" yWindow="2430" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>CAS Number</t>
   </si>
@@ -84,12 +85,15 @@
   </si>
   <si>
     <t>100038-54-8</t>
+  </si>
+  <si>
+    <t>drdrtrdt</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -448,7 +452,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -537,7 +541,12 @@
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="1"/>
+      <c r="A11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11">
+        <v>4564564</v>
+      </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>

</xml_diff>